<commit_message>
Amber : P : RP : add taxi sheet in Wiesbaden.xlsx
</commit_message>
<xml_diff>
--- a/P(Path)/RP(Rhine-Path)/RheinWegDE/RheinWeg-Beispiel-Firma-14-10-2026.xlsx
+++ b/P(Path)/RP(Rhine-Path)/RheinWegDE/RheinWeg-Beispiel-Firma-14-10-2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr filterPrivacy="1"/>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1EFE4AA-0D62-C145-910E-1CCA2D94C806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9360" yWindow="14720" windowWidth="36820" windowHeight="16520" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9360" yWindow="14720" windowWidth="36820" windowHeight="16520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" Inhaltsverzeichnis" sheetId="1" r:id="rId1"/>
@@ -835,6 +835,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -853,15 +862,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1209,50 +1209,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="13" t="s">
         <v>213</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="8" t="s">
+      <c r="B1" s="14"/>
+      <c r="C1" s="15" t="s">
         <v>214</v>
       </c>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="9"/>
-      <c r="T1" s="9"/>
-      <c r="U1" s="9"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="16"/>
+      <c r="T1" s="16"/>
+      <c r="U1" s="16"/>
     </row>
     <row r="2" spans="1:21" ht="19" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
     </row>
     <row r="3" spans="1:21" ht="26.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="5" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1380,29 +1380,29 @@
     <col min="8" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="15" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:8" s="9" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>189</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="11" t="s">
         <v>193</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="H1" s="11" t="s">
         <v>196</v>
       </c>
     </row>
@@ -1450,20 +1450,20 @@
     <col min="5" max="5" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="15" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:5" s="9" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="11" t="s">
         <v>206</v>
       </c>
     </row>
@@ -1502,20 +1502,20 @@
     <col min="5" max="5" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="15" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:5" s="9" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="11" t="s">
         <v>206</v>
       </c>
     </row>
@@ -1547,12 +1547,12 @@
   <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="26.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20" style="13" customWidth="1"/>
+    <col min="1" max="1" width="20" style="7" customWidth="1"/>
     <col min="2" max="2" width="100" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1560,7 +1560,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1568,7 +1568,7 @@
       </c>
     </row>
     <row r="3" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="6" t="s">
         <v>19</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1576,7 +1576,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -1584,7 +1584,7 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -1592,7 +1592,7 @@
       </c>
     </row>
     <row r="6" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="6" t="s">
         <v>24</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -1600,7 +1600,7 @@
       </c>
     </row>
     <row r="7" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="6" t="s">
         <v>26</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -1608,7 +1608,7 @@
       </c>
     </row>
     <row r="8" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="6" t="s">
         <v>28</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -1616,7 +1616,7 @@
       </c>
     </row>
     <row r="9" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -1624,7 +1624,7 @@
       </c>
     </row>
     <row r="10" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -1632,7 +1632,7 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="6" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -1640,7 +1640,7 @@
       </c>
     </row>
     <row r="12" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="6" t="s">
         <v>34</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -1648,7 +1648,7 @@
       </c>
     </row>
     <row r="13" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="6" t="s">
         <v>36</v>
       </c>
       <c r="B13" s="1" t="s">
@@ -1656,7 +1656,7 @@
       </c>
     </row>
     <row r="14" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -1664,7 +1664,7 @@
       </c>
     </row>
     <row r="15" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="6" t="s">
         <v>40</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -1672,7 +1672,7 @@
       </c>
     </row>
     <row r="16" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1680,7 +1680,7 @@
       </c>
     </row>
     <row r="17" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="6" t="s">
         <v>43</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -1688,7 +1688,7 @@
       </c>
     </row>
     <row r="18" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="6" t="s">
         <v>44</v>
       </c>
       <c r="B18" s="1" t="s">
@@ -1696,7 +1696,7 @@
       </c>
     </row>
     <row r="19" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="6" t="s">
         <v>46</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -1704,7 +1704,7 @@
       </c>
     </row>
     <row r="20" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="6" t="s">
         <v>48</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -1712,7 +1712,7 @@
       </c>
     </row>
     <row r="21" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="6" t="s">
         <v>49</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -1720,7 +1720,7 @@
       </c>
     </row>
     <row r="22" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="6" t="s">
         <v>51</v>
       </c>
       <c r="B22" s="1" t="s">
@@ -1728,7 +1728,7 @@
       </c>
     </row>
     <row r="23" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="6" t="s">
         <v>53</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -1736,7 +1736,7 @@
       </c>
     </row>
     <row r="24" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="6" t="s">
         <v>55</v>
       </c>
       <c r="B24" s="1" t="s">
@@ -1744,7 +1744,7 @@
       </c>
     </row>
     <row r="25" spans="1:2" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="6" t="s">
         <v>56</v>
       </c>
       <c r="B25" s="1" t="s">
@@ -1767,26 +1767,26 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="15" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+    <row r="2" spans="1:7" s="9" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1838,17 +1838,17 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="15" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+    <row r="2" spans="1:4" s="9" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="8" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1895,7 +1895,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="5" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="19" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="5" t="s">
         <v>91</v>
       </c>
     </row>
@@ -2037,7 +2037,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="19" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="5" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       </c>
     </row>
     <row r="30" spans="1:3" ht="19" x14ac:dyDescent="0.25">
-      <c r="A30" s="11" t="s">
+      <c r="A30" s="5" t="s">
         <v>125</v>
       </c>
     </row>
@@ -2245,7 +2245,7 @@
       </c>
     </row>
     <row r="32" spans="1:3" ht="19" x14ac:dyDescent="0.25">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="5" t="s">
         <v>128</v>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
       </c>
     </row>
     <row r="37" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A37" s="11" t="s">
+      <c r="A37" s="5" t="s">
         <v>137</v>
       </c>
     </row>
@@ -2337,7 +2337,7 @@
       </c>
     </row>
     <row r="39" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A39" s="11" t="s">
+      <c r="A39" s="5" t="s">
         <v>146</v>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
     </row>
     <row r="41" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A41" s="11" t="s">
+      <c r="A41" s="5" t="s">
         <v>150</v>
       </c>
     </row>
@@ -2392,17 +2392,17 @@
     <col min="2" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="13" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:4" s="7" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="10" t="s">
         <v>157</v>
       </c>
     </row>
@@ -2465,40 +2465,40 @@
     <col min="5" max="6" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="15" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:6" s="9" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="11" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="10">
+      <c r="A2" s="17">
         <v>1</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="17" t="s">
         <v>215</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="17" t="s">
         <v>169</v>
       </c>
       <c r="F2" t="s">
@@ -2506,11 +2506,11 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="10"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
+      <c r="A3" s="17"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
       <c r="F3" t="s">
         <v>171</v>
       </c>
@@ -2557,25 +2557,25 @@
     <col min="4" max="4" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="15" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:4" s="9" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>174</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="11" t="s">
         <v>176</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="11" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="17" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="17" t="s">
         <v>64</v>
       </c>
       <c r="C2" t="s">
@@ -2605,34 +2605,34 @@
         <v>179</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="15" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:5" s="9" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="11" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="17" t="s">
         <v>215</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="17" t="s">
         <v>184</v>
       </c>
       <c r="E3" t="s">
@@ -2644,37 +2644,37 @@
         <v>185</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="15" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
+    <row r="7" spans="1:5" s="9" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="11" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="17" t="s">
         <v>215</v>
       </c>
       <c r="B8" t="s">
         <v>217</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="17" t="s">
         <v>188</v>
       </c>
     </row>

</xml_diff>